<commit_message>
Ajout de la page StructureDefinition-Auteur-into.md 6c07ae780b07cf6f3c1b16516ceac62381508e1f
</commit_message>
<xml_diff>
--- a/HTR-IGDoc/ig/StructureDefinition-Auteur.xlsx
+++ b/HTR-IGDoc/ig/StructureDefinition-Auteur.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-23T14:02:58+00:00</t>
+    <t>2025-02-24T10:33:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,47 +81,8 @@
     <t>Description</t>
   </si>
   <si>
-    <t xml:space="preserve">Auteur du document : ce peut être un professionnel, un patient/usager ou un système. 
-- Pour un professionnel ou un système, la structure de rattachement doit être précisée.
-  Voici les cas d'usage des documents et leurs auteurs :
-  &lt;table&gt;
-    &lt;tr&gt;
-      &lt;th&gt;Cas d'usage&lt;/th&gt;
-      &lt;th&gt;Auteur(s) du document&lt;/th&gt;
-      &lt;th&gt;Structure de l'auteur&lt;/th&gt;
-    &lt;/tr&gt;
-    &lt;tr&gt;
-      &lt;td&gt;Création d'un document par un professionnel sur son logiciel professionnel&lt;/td&gt;
-      &lt;td&gt;Professionnel&lt;/td&gt;
-      &lt;td&gt;Structure&lt;/td&gt;
-    &lt;/tr&gt;
-    &lt;tr&gt;
-      &lt;td&gt;Création d'un document patient par un professionnel sur son logiciel professionnel pour le compte du patient&lt;/td&gt;
-      &lt;td&gt;Professionnel&lt;/td&gt;
-      &lt;td&gt;Structure&lt;/td&gt;
-    &lt;/tr&gt;
-    &lt;tr&gt;
-      &lt;td&gt;Création d'un document patient par le patient&lt;/td&gt;
-      &lt;td&gt;Patient&lt;/td&gt;
-      &lt;td&gt;non utilisé&lt;/td&gt;
-    &lt;/tr&gt;
-    &lt;tr&gt;
-      &lt;td&gt;Création d'un document par un système (dispositif, automate, …) de structure (ES, …)&lt;/td&gt;
-      &lt;td&gt;Système de structure&lt;/td&gt;
-      &lt;td&gt;Structure&lt;/td&gt;
-    &lt;/tr&gt;
-    &lt;tr&gt;
-      &lt;td&gt;Création d'un document par un Service numérique référencé (SNR)&lt;/td&gt;
-      &lt;td&gt;SNR&lt;/td&gt;
-      &lt;td&gt;Editeur&lt;/td&gt;
-    &lt;/tr&gt;
-    &lt;tr&gt;
-      &lt;td&gt;Création d'un document par le DP&lt;/td&gt;
-      &lt;td&gt;CNOP/DP&lt;/td&gt;
-      &lt;td&gt;CNOP&lt;/td&gt;
-    &lt;/tr&gt;
-  &lt;/table&gt;
-</t>
+    <t>Auteur du document : ce peut être un professionnel, un patient/usager ou un système. 
+- Pour un professionnel ou un système, la structure de rattachement doit être précisée.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>